<commit_message>
update pmr ciclo oct
</commit_message>
<xml_diff>
--- a/PMR_Historico.xlsx
+++ b/PMR_Historico.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CR-L1152" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CR-L1156" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CR-L1157" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyeccion" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +40,9 @@
       <color rgb="FFE2E8F0"/>
     </font>
     <font/>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -65,13 +69,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1115,6 +1123,567 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Proyección PMR al cierre del año — seguimiento según el último informe de ciclo PMR (se reemplaza en cada informe)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Operación</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Corte del seguimiento</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Calificación sistema al corte (parcial)</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>SI al corte</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Calificación proyectada cierre 2026</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Condición / supuesto</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>¿Mejora factible?</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Comentarios de seguimiento</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Plan de acción</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>CR-L1032</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Primer período enero-junio 2026</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Informe ciclo PMR oct-2026 (versión final rev2)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Problema</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Problema</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Desembolsar ≥US$29mn antes del 13-nov-2026 (último desembolso) la llevaría a alerta (2,0); lo planeado en el sistema es un desembolso de US$12mn en noviembre.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Solo a alerta. Satisfactorio no factible (requiere ≈US$95mn de valor ganado).</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Desembolsos en problema (0,77) y SPI(a)/CPI(a) en alerta (0,54/0,69) por las metas 2026 de Barranca–Limonal y RN-35. No existe escenario factible para satisfactorio en 2026.</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Solicitar al TL corregir la cifra de desembolso (80% vs. 77,3% en sistema) y formalizar la prórroga antes del 13-nov-2026. Ajustar las metas 2027 antes de su bloqueo en marzo 2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>CR-L1065</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Primer período enero-junio 2026</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Informe ciclo PMR oct-2026 (versión final rev2)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Satisfactorio</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Satisfactorio</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Se mantiene aun si supera 19,6 meses desde el 95% desembolsado (SI 2,6).</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Ya satisfactoria; no requiere mejora.</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Operación en cierre (100% desembolsado). Meses tras 95% desembolsado = 12 (alerta), sin efecto en la calificación global.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Completar el cierre administrativo y el PCR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>CR-L1139</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Primer período enero-junio 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Informe ciclo PMR oct-2026 (versión final rev2)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Satisfactorio</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Satisfactorio</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Evitar más de US$17mn de gasto sin avance reconocido (2,7) y nunca más de US$42mn (alerta, 2,4).</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Ya satisfactoria; no requiere mejora.</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Sin riesgo de cambio en 2026: el desembolso (73%) supera el benchmark de diciembre (66,5%). La probabilidad bajó a Media, consistente con el plazo del corredor San José–San Ramón.</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Avanzar la modificación de la MR y dar seguimiento a expropiaciones de Naranjo (Lote #4). Iniciar en el I semestre 2027 el trámite de prórroga (vence 29-sep-2027).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>CR-L1151</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Primer período enero-junio 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Informe ciclo PMR oct-2026 (versión final rev2)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Alerta</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Satisfactorio</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Reportar como gasto los US$13,2mn justificados a sep-2026 (≥US$5,7mn adicionales en Punta Sur): SPI(a) ≈0,84 y SI 2,5; con el desembolso de US$10mn en análisis, SI 2,6.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Sí, condicionado a reportar la ejecución de Punta Sur del II semestre.</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Sin acciones cierra 2026 en alerta (2,2): el indicador de desembolsos cae a problema con el benchmark de diciembre.</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Confirmar con el TL la ejecución de Punta Sur del II semestre. Definir el financiamiento del Tramo Central (recursos nacionales) y la modificación de MR/reasignación; formalizar la nueva fecha de la evaluación intermedia (venció jul-2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>CR-L1137</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Primer período enero-junio 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Informe ciclo PMR oct-2026 (versión final rev2)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Satisfactorio</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Satisfactorio</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Registrar en diciembre las 3 DP entregadas en jul-ago lleva el SI a 3,0. Más de US$3,9mn de pagos sin avance reconocido la llevaría a alerta (2,4).</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Sí (2,7 → 3,0) con hechos ya ocurridos y valores planeados.</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Mejora frente a 2025 (alerta con override) por la entrega de 5 DP y 1 CCP. Margen estrecho en CPI(a).</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Atender las salvaguardas en "Insatisfactorio", la rescisión del contratista de 4 CCP y la prórroga del plazo (vence 17-mar-2027).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>CR-J0002</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Primer período enero-junio 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Informe ciclo PMR oct-2026 (versión final rev2)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Alerta</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Alerta</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>No superar US$0,3mn de gasto sin avance reconocido en productos con meta física (si no, problema 1,95).</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>No factible mejorar más allá de alerta en 2026.</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Mejora frente a 2025 (problema). SPI (0,06) y SPI(a) (0,26) siguen en problema; hay escenarios teóricos para satisfactorio, pero ninguno factible en 2026 (CCP Upala no se ejecutará).</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Tramitar la prórroga (vence 5-abr-2027) junto con la reasignación de CIS Mora y CATEM Sur. Evaluación intermedia vence 31-oct-2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>CR-L1152</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Primer período enero-junio 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Informe ciclo PMR oct-2026 (versión final rev2)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Alerta (etapa 1)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Satisfactorio (con override)</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Sin ratificación al 31-dic el sistema la calificaría en problema (756 días); se propone mantenerla satisfactoria aplicando override de la calificación del sistema. Con ratificación y vigencia antes del corte y elegibilidad en ≤73 días → satisfactorio.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>No con parámetros del PMR; depende de la Asamblea Legislativa.</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Etapa 1: al 30-jun-2026 sumaba 572 días desde la aprobación; superó el umbral de problema (626,5 días) el 23-ago-2026. Solo la ratificación y vigencia antes del corte cambia el indicador.</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Solicitar al TL una actualización del trámite en la comisión de Hacendarios, la posición del nuevo Gobierno y una fecha estimada de ratificación. Preparar las condiciones de elegibilidad para cumplirlas en ≤73 días tras la vigencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>CR-L1156</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Primer período enero-junio 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Informe ciclo PMR oct-2026 (versión final rev2)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Sin clasificación</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Sin clasificación</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Si el sistema muestra calificación: alerta al 31-dic (554 días) y problema desde el 13-mar-2027. Con ratificación y vigencia antes del corte → satisfactorio.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>No con parámetros del PMR; depende de la Asamblea Legislativa.</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>El sistema sigue sin semáforo ("for tracking purpose only"). Etapa 1: al 30-jun-2026 sumaba 370 días desde la aprobación (25-jun-2025); el umbral de alerta (375 días) se cruzó el 5-jul-2026.</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Consultar a SPD y actualizar el estado de la ratificación con el nuevo Gobierno. Override sería la única opción de mantenerla satisfactoria sin ratificación, en caso que el sistema muestre calificación en el ciclo de marzo 2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>CR-L1157</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Primer período enero-junio 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Informe ciclo PMR oct-2026 (versión final rev2)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Alerta (etapa 1)</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Satisfactorio (con ajuste del plan inicial)</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Ajustar las metas 2026 del plan inicial (P y P(a)) a los pagos efectivos antes del ciclo de marzo 2027 → SI 2,7–3,0. Sin ajuste: con pagos ≥US$7,9mn → 2,55; con pagos menores → alerta (2,1); sin pagos → problema (1,2).</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Sí: el ajuste del plan inicial antes de marzo 2027 la deja en satisfactorio.</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Alcanzó la elegibilidad el 6-oct-2026 (180 días desde la vigencia); pasa a etapa 2 y su calificación 2026 dependerá del ajuste del plan inicial.</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Acordar con el TL y el ICE el ajuste de las metas del plan inicial (2026 y 2027) antes de marzo 2027, con un plan de pagos realista (anticipo de reactores de US$1,8mn, LPI de la PHVG y LPI de luminarias LED). Ajustar también la MR del Componente 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>CR-L1066</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Informe ciclo PMR oct-2026 (versión final rev2)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Operación finalizada; no forma parte del ciclo PMR de oct-2026.</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>